<commit_message>
Updated file names for Iwaniuk 2001
</commit_message>
<xml_diff>
--- a/Iwaniuk_etal_2001/Iwaniuk_etal_2001_table2_snapshot.xlsx
+++ b/Iwaniuk_etal_2001/Iwaniuk_etal_2001_table2_snapshot.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MILONI\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/crossmodal/Library/CloudStorage/OneDrive-AllenInstitute/Species/Evo-M1-Trait-Data/Iwaniuk_etal_2001/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{43116703-0C3F-4670-9237-AD9CEDC87979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0EF22B6-1EA7-F543-BBEE-36B88DD73D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8820" yWindow="0" windowWidth="10420" windowHeight="10640"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="16900" windowHeight="20360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Iwaniuk_etal_2001_table1_snapsh" sheetId="1" r:id="rId1"/>
@@ -124,7 +124,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.000"/>
+  </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -619,21 +622,23 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -693,9 +698,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -733,7 +738,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -839,7 +844,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -981,73 +986,69 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.1796875" customWidth="1"/>
-    <col min="2" max="2" width="17.6328125" customWidth="1"/>
-    <col min="3" max="3" width="17.26953125" customWidth="1"/>
-    <col min="4" max="4" width="17.36328125" customWidth="1"/>
-    <col min="5" max="5" width="17.26953125" customWidth="1"/>
-    <col min="6" max="6" width="16.90625" customWidth="1"/>
-    <col min="7" max="7" width="17.08984375" customWidth="1"/>
+    <col min="1" max="6" width="18.1640625" customWidth="1"/>
+    <col min="7" max="7" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>9</v>
       </c>
+      <c r="B6" s="6"/>
       <c r="C6">
         <v>0</v>
       </c>
@@ -1060,14 +1061,15 @@
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="7">
         <v>-5.7000000000000002E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>32</v>
       </c>
+      <c r="B7" s="6"/>
       <c r="C7">
         <v>0</v>
       </c>
@@ -1080,14 +1082,15 @@
       <c r="F7">
         <v>1</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="7">
         <v>-7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>10</v>
       </c>
+      <c r="B8" s="6"/>
       <c r="C8">
         <v>1</v>
       </c>
@@ -1100,14 +1103,15 @@
       <c r="F8">
         <v>3</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="7">
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>11</v>
       </c>
+      <c r="B9" s="6"/>
       <c r="C9">
         <v>1</v>
       </c>
@@ -1120,15 +1124,15 @@
       <c r="F9">
         <v>2</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="7">
         <v>-0.14499999999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>12</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="6">
         <v>0.38</v>
       </c>
       <c r="C10">
@@ -1143,15 +1147,15 @@
       <c r="F10">
         <v>2</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="7">
         <v>-3.3000000000000002E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>13</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="6">
         <v>0.75</v>
       </c>
       <c r="C11">
@@ -1166,14 +1170,15 @@
       <c r="F11">
         <v>2</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="7">
         <v>-0.151</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>14</v>
       </c>
+      <c r="B12" s="6"/>
       <c r="C12">
         <v>1</v>
       </c>
@@ -1186,15 +1191,15 @@
       <c r="F12">
         <v>1</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="7">
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>15</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="6">
         <v>0.13</v>
       </c>
       <c r="C13">
@@ -1209,15 +1214,15 @@
       <c r="F13">
         <v>2</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="7">
         <v>-0.113</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>16</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="6">
         <v>0.31</v>
       </c>
       <c r="C14">
@@ -1232,15 +1237,15 @@
       <c r="F14">
         <v>1</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="7">
         <v>-0.152</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>17</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="6">
         <v>0.5</v>
       </c>
       <c r="C15">
@@ -1255,14 +1260,15 @@
       <c r="F15">
         <v>2</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="7">
         <v>-0.22900000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>18</v>
       </c>
+      <c r="B16" s="6"/>
       <c r="C16">
         <v>1</v>
       </c>
@@ -1275,15 +1281,15 @@
       <c r="F16">
         <v>1</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="7">
         <v>-9.4E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>19</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="6">
         <v>0.13</v>
       </c>
       <c r="C17">
@@ -1298,15 +1304,15 @@
       <c r="F17">
         <v>2</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="7">
         <v>-9.4E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>20</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="6">
         <v>0.13</v>
       </c>
       <c r="C18">
@@ -1321,15 +1327,15 @@
       <c r="F18">
         <v>2</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="7">
         <v>0.114</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>21</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="6">
         <v>0.13</v>
       </c>
       <c r="C19">
@@ -1344,14 +1350,15 @@
       <c r="F19">
         <v>0</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="7">
         <v>0.13400000000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>22</v>
       </c>
+      <c r="B20" s="6"/>
       <c r="C20">
         <v>1</v>
       </c>
@@ -1364,15 +1371,15 @@
       <c r="F20">
         <v>1</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="7">
         <v>-1.2E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>23</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="6">
         <v>0.44</v>
       </c>
       <c r="C21">
@@ -1387,14 +1394,15 @@
       <c r="F21">
         <v>1</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="7">
         <v>6.8000000000000005E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>24</v>
       </c>
+      <c r="B22" s="6"/>
       <c r="C22">
         <v>0</v>
       </c>
@@ -1407,15 +1415,15 @@
       <c r="F22">
         <v>0</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="7">
         <v>-3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>25</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="6">
         <v>0.38</v>
       </c>
       <c r="C23">
@@ -1430,15 +1438,15 @@
       <c r="F23">
         <v>1</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="7">
         <v>-1.6E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>26</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="6">
         <v>0.31</v>
       </c>
       <c r="C24">
@@ -1453,15 +1461,15 @@
       <c r="F24">
         <v>1</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="7">
         <v>-0.182</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>27</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="6">
         <v>0</v>
       </c>
       <c r="C25">
@@ -1476,15 +1484,15 @@
       <c r="F25">
         <v>0</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="7">
         <v>4.1000000000000002E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>28</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="6">
         <v>0</v>
       </c>
       <c r="C26">
@@ -1499,15 +1507,15 @@
       <c r="F26">
         <v>0</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="7">
         <v>0.09</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>29</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="6">
         <v>0.94</v>
       </c>
       <c r="C27">
@@ -1522,14 +1530,15 @@
       <c r="F27">
         <v>4</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="7">
         <v>-0.104</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>30</v>
       </c>
+      <c r="B28" s="6"/>
       <c r="C28">
         <v>1</v>
       </c>
@@ -1542,11 +1551,11 @@
       <c r="F28">
         <v>4</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="7">
         <v>4.4999999999999998E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>31</v>
       </c>
@@ -1565,4 +1574,283 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="66af2654134d243f62aac8e2b322f1d6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2bc3adf68671d86faa9c37249f400344" ns2:_="" ns3:_="">
+    <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <xsd:import namespace="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="11" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="12" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="13" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="16" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="20" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2a91012f-191a-4297-80da-223551dc3c4f" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="22" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="17" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="18" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{ec99e049-fb75-4c8f-a4b4-b132771b9bd6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4520FAFC-1D95-44A4-A356-BEF761B55D4E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8702C5BB-2F4E-4DDB-B3E7-DEB08B72B654}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>